<commit_message>
Tokens en Variables de Sistema
Se quita el archivo .env y se modifica el código para tomar los tokens de las plataformas de variables de sistema.
</commit_message>
<xml_diff>
--- a/output/consulta_validacion.xlsx
+++ b/output/consulta_validacion.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q42"/>
+  <dimension ref="A1:Q65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -428,8 +428,8 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="27" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="33" customWidth="1" min="6" max="6"/>
-    <col width="33" customWidth="1" min="7" max="7"/>
+    <col width="39" customWidth="1" min="6" max="6"/>
+    <col width="39" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
@@ -527,22 +527,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SPRING</t>
+          <t>ROOMI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>7018044981357</t>
+          <t>6767608267011</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6259</t>
+          <t>1159</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2025-11-21T23:22:33-06:00</t>
+          <t>2025-11-27T14:47:34-06:00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -552,12 +552,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>FABIOLA JERALDINNE CRUZ GARDUÑO</t>
+          <t>CELIA DELGADO AGUIÑAGA</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>FABIOLA JERALDINNE CRUZ GARDUÑO</t>
+          <t>CELIA DELGADO AGUIÑAGA</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -573,19 +573,19 @@
         <v>2</v>
       </c>
       <c r="L2" t="n">
-        <v>979</v>
+        <v>1499</v>
       </c>
       <c r="M2" t="n">
-        <v>979.01</v>
+        <v>1499.01</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>19.4941617,-99.03467649999999</t>
+          <t>21.8984234,-102.2518749</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>19.4941617,-99.03467649999999</t>
+          <t>21.8984234,-102.2518749</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>SPRING_6259</t>
+          <t>ROOMI_1159</t>
         </is>
       </c>
     </row>
@@ -607,17 +607,17 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>7018002514029</t>
+          <t>7036876882029</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>6258</t>
+          <t>6497</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>2025-11-21T23:08:54-06:00</t>
+          <t>2025-11-27T23:56:47-06:00</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
@@ -627,12 +627,12 @@
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>JONATHAN SILVA</t>
+          <t>ERNESTO VELAZQUEZ CUELLAR</t>
         </is>
       </c>
       <c r="G3" s="1" t="inlineStr">
         <is>
-          <t>JONATHAN SILVA</t>
+          <t>ERNESTO VELAZQUEZ CUELLAR</t>
         </is>
       </c>
       <c r="H3" s="1" t="n">
@@ -648,29 +648,29 @@
         <v>2</v>
       </c>
       <c r="L3" s="1" t="n">
-        <v>6696.55</v>
+        <v>26522.1</v>
       </c>
       <c r="M3" s="1" t="n">
-        <v>6696.56</v>
+        <v>26522.11</v>
       </c>
       <c r="N3" s="1" t="inlineStr">
         <is>
-          <t>29.0857259,-111.0506463</t>
+          <t>19.9001399,-99.34451109999999</t>
         </is>
       </c>
       <c r="O3" s="1" t="inlineStr">
         <is>
-          <t>29.0857259,-111.0506463</t>
+          <t>19.9001399,-99.34451109999999</t>
         </is>
       </c>
       <c r="P3" s="1" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>ENCONTRADO DÍA SIGUIENTE</t>
         </is>
       </c>
       <c r="Q3" s="1" t="inlineStr">
         <is>
-          <t>SPRING_6258</t>
+          <t>SPRING_6497</t>
         </is>
       </c>
     </row>
@@ -682,17 +682,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>7017940287597</t>
+          <t>7036698591341</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>6257</t>
+          <t>6496</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2025-11-21T22:41:33-06:00</t>
+          <t>2025-11-27T22:38:23-06:00</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -702,40 +702,40 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>RONAN OBED HERNÁNDEZ DAMIÁN</t>
+          <t>ARELI QUEZADA</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>RONAN OBED HERNÁNDEZ DAMIÁN</t>
+          <t>ARELI QUEZADA</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L4" t="n">
-        <v>15418</v>
+        <v>18944.1</v>
       </c>
       <c r="M4" t="n">
-        <v>15418.01</v>
+        <v>18944.11</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>17.1186814,-96.7561202</t>
+          <t>21.9187226,-102.3262697</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>17.1186814,-96.7561202</t>
+          <t>21.9187226,-102.3262697</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -745,7 +745,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>SPRING_6257</t>
+          <t>SPRING_6496</t>
         </is>
       </c>
     </row>
@@ -757,17 +757,17 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>7017873408109</t>
+          <t>7036680306797</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>6256</t>
+          <t>6495</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>2025-11-21T22:05:03-06:00</t>
+          <t>2025-11-27T22:25:47-06:00</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
@@ -777,40 +777,40 @@
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>DORA EVELIA PASOS RIVERA</t>
+          <t>JUAN ROMERO</t>
         </is>
       </c>
       <c r="G5" s="1" t="inlineStr">
         <is>
-          <t>DORA EVELIA PASOS RIVERA</t>
+          <t>JUAN ROMERO</t>
         </is>
       </c>
       <c r="H5" s="1" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I5" s="1" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J5" s="1" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K5" s="1" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L5" s="1" t="n">
-        <v>5399</v>
+        <v>17340.3</v>
       </c>
       <c r="M5" s="1" t="n">
-        <v>5399.01</v>
+        <v>17340.31</v>
       </c>
       <c r="N5" s="1" t="inlineStr">
         <is>
-          <t>19.8764259,-97.5880785</t>
+          <t>19.4948576,-99.2353675</t>
         </is>
       </c>
       <c r="O5" s="1" t="inlineStr">
         <is>
-          <t>19.8764259,-97.5880785</t>
+          <t>19.4948576,-99.2353675</t>
         </is>
       </c>
       <c r="P5" s="1" t="inlineStr">
@@ -820,7 +820,7 @@
       </c>
       <c r="Q5" s="1" t="inlineStr">
         <is>
-          <t>SPRING_6256</t>
+          <t>SPRING_6495</t>
         </is>
       </c>
     </row>
@@ -832,17 +832,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>7017847750765</t>
+          <t>7036678340717</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>6255</t>
+          <t>6494</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2025-11-21T21:50:18-06:00</t>
+          <t>2025-11-27T22:24:27-06:00</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -852,12 +852,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>CRISTINA TORAL MORA</t>
+          <t>JORGE CRUZ ORTEGA</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>CRISTINA TORAL MORA</t>
+          <t>JORGE CRUZ ORTEGA</t>
         </is>
       </c>
       <c r="H6" t="n">
@@ -873,19 +873,19 @@
         <v>2</v>
       </c>
       <c r="L6" t="n">
-        <v>12309</v>
+        <v>499</v>
       </c>
       <c r="M6" t="n">
-        <v>12309.01</v>
+        <v>499.01</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>19.1826927,-96.13791619999999</t>
+          <t>25.7197798,-100.2593136</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>19.1826927,-96.13791619999999</t>
+          <t>25.7197798,-100.2593136</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -895,7 +895,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>SPRING_6255</t>
+          <t>SPRING_6494</t>
         </is>
       </c>
     </row>
@@ -907,17 +907,17 @@
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>7017775071341</t>
+          <t>7036625387629</t>
         </is>
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>6253</t>
+          <t>6493</t>
         </is>
       </c>
       <c r="D7" s="1" t="inlineStr">
         <is>
-          <t>2025-11-21T21:08:56-06:00</t>
+          <t>2025-11-27T22:06:38-06:00</t>
         </is>
       </c>
       <c r="E7" s="1" t="inlineStr">
@@ -927,12 +927,12 @@
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>PAOLA GUTIERREZ ORTIZ</t>
+          <t>MARIA DE LA LUZ PICHARDO GÓMEZ</t>
         </is>
       </c>
       <c r="G7" s="1" t="inlineStr">
         <is>
-          <t>PAOLA GUTIERREZ ORTIZ</t>
+          <t>MARIA DE LA LUZ PICHARDO GÓMEZ</t>
         </is>
       </c>
       <c r="H7" s="1" t="n">
@@ -948,19 +948,19 @@
         <v>2</v>
       </c>
       <c r="L7" s="1" t="n">
-        <v>8099</v>
+        <v>999</v>
       </c>
       <c r="M7" s="1" t="n">
-        <v>8099.01</v>
+        <v>999.01</v>
       </c>
       <c r="N7" s="1" t="inlineStr">
         <is>
-          <t>19.5810159,-96.93773949999999</t>
+          <t>19.5239774,-99.1753052</t>
         </is>
       </c>
       <c r="O7" s="1" t="inlineStr">
         <is>
-          <t>19.5810159,-96.93773949999999</t>
+          <t>19.5239774,-99.1753052</t>
         </is>
       </c>
       <c r="P7" s="1" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="Q7" s="1" t="inlineStr">
         <is>
-          <t>SPRING_6253</t>
+          <t>SPRING_6493</t>
         </is>
       </c>
     </row>
@@ -982,17 +982,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>7017755902061</t>
+          <t>7036614869101</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>6252</t>
+          <t>6492</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2025-11-21T21:02:19-06:00</t>
+          <t>2025-11-27T22:03:06-06:00</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1002,12 +1002,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>ESMERALDA ARELLANO LOZANO</t>
+          <t>EMILY ITHAYETZI SANTOS VARGAS</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>ESMERALDA ARELLANO LOZANO</t>
+          <t>EMILY ITHAYETZI SANTOS VARGAS</t>
         </is>
       </c>
       <c r="H8" t="n">
@@ -1023,19 +1023,19 @@
         <v>2</v>
       </c>
       <c r="L8" t="n">
-        <v>3799</v>
+        <v>1699</v>
       </c>
       <c r="M8" t="n">
-        <v>3799.01</v>
+        <v>1699.01</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>19.3208959,-99.2564953</t>
+          <t>17.0651999,-96.69392189999999</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>19.3208959,-99.2564953</t>
+          <t>17.0651999,-96.69392189999999</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -1045,7 +1045,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>SPRING_6252</t>
+          <t>SPRING_6492</t>
         </is>
       </c>
     </row>
@@ -1057,17 +1057,17 @@
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
-          <t>7017675685997</t>
+          <t>7036580986989</t>
         </is>
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>6251</t>
+          <t>6491</t>
         </is>
       </c>
       <c r="D9" s="1" t="inlineStr">
         <is>
-          <t>2025-11-21T20:17:12-06:00</t>
+          <t>2025-11-27T21:45:06-06:00</t>
         </is>
       </c>
       <c r="E9" s="1" t="inlineStr">
@@ -1077,40 +1077,40 @@
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>ELIZABETH AGUAYO</t>
+          <t>NORMA HERNANDEZ MORENO</t>
         </is>
       </c>
       <c r="G9" s="1" t="inlineStr">
         <is>
-          <t>ELIZABETH AGUAYO</t>
+          <t>NORMA HERNANDEZ MORENO</t>
         </is>
       </c>
       <c r="H9" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I9" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J9" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K9" s="1" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L9" s="1" t="n">
-        <v>12786.16</v>
+        <v>3899</v>
       </c>
       <c r="M9" s="1" t="n">
-        <v>12786.17</v>
+        <v>3899.01</v>
       </c>
       <c r="N9" s="1" t="inlineStr">
         <is>
-          <t>23.1007288,-109.7147539</t>
+          <t>19.3947041,-99.1769709</t>
         </is>
       </c>
       <c r="O9" s="1" t="inlineStr">
         <is>
-          <t>23.1007288,-109.7147539</t>
+          <t>19.3947041,-99.1769709</t>
         </is>
       </c>
       <c r="P9" s="1" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="Q9" s="1" t="inlineStr">
         <is>
-          <t>SPRING_6251</t>
+          <t>SPRING_6491</t>
         </is>
       </c>
     </row>
@@ -1132,17 +1132,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>7017669984365</t>
+          <t>7036464726125</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>6250</t>
+          <t>6490</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2025-11-21T20:15:23-06:00</t>
+          <t>2025-11-27T20:58:24-06:00</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1152,12 +1152,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>SANTIAGO GARCÍA SUAREZ</t>
+          <t>ANA KARINA SEGURA</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>SANTIAGO GARCÍA SUAREZ</t>
+          <t>ANA KARINA SEGURA</t>
         </is>
       </c>
       <c r="H10" t="n">
@@ -1173,19 +1173,19 @@
         <v>2</v>
       </c>
       <c r="L10" t="n">
-        <v>8074.05</v>
+        <v>13733.1</v>
       </c>
       <c r="M10" t="n">
-        <v>8074.06</v>
+        <v>13733.11</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>19.2677752,-98.99775299999999</t>
+          <t>22.1391478,-100.9289876</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>19.2677752,-98.99775299999999</t>
+          <t>22.1391478,-100.9289876</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>SPRING_6250</t>
+          <t>SPRING_6490</t>
         </is>
       </c>
     </row>
@@ -1207,17 +1207,17 @@
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
-          <t>7017499426925</t>
+          <t>7036448833645</t>
         </is>
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>6249</t>
+          <t>6489</t>
         </is>
       </c>
       <c r="D11" s="1" t="inlineStr">
         <is>
-          <t>2025-11-21T19:07:22-06:00</t>
+          <t>2025-11-27T20:50:03-06:00</t>
         </is>
       </c>
       <c r="E11" s="1" t="inlineStr">
@@ -1227,12 +1227,12 @@
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>LUCERO LOPEZ GUTIERREZ</t>
+          <t>EMMANUEL ALEJANDRO RIVERA PÉREZ</t>
         </is>
       </c>
       <c r="G11" s="1" t="inlineStr">
         <is>
-          <t>LUCERO LOPEZ GUTIERREZ</t>
+          <t>EMMANUEL ALEJANDRO RIVERA PÉREZ</t>
         </is>
       </c>
       <c r="H11" s="1" t="n">
@@ -1248,19 +1248,19 @@
         <v>3</v>
       </c>
       <c r="L11" s="1" t="n">
-        <v>25603.2</v>
+        <v>5048</v>
       </c>
       <c r="M11" s="1" t="n">
-        <v>25603.21</v>
+        <v>5048.01</v>
       </c>
       <c r="N11" s="1" t="inlineStr">
         <is>
-          <t>19.293337,-99.14478229999999</t>
+          <t>19.487499,-96.8013612</t>
         </is>
       </c>
       <c r="O11" s="1" t="inlineStr">
         <is>
-          <t>19.293337,-99.14478229999999</t>
+          <t>19.487499,-96.8013612</t>
         </is>
       </c>
       <c r="P11" s="1" t="inlineStr">
@@ -1270,7 +1270,7 @@
       </c>
       <c r="Q11" s="1" t="inlineStr">
         <is>
-          <t>SPRING_6249</t>
+          <t>SPRING_6489</t>
         </is>
       </c>
     </row>
@@ -1282,17 +1282,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>7017428484205</t>
+          <t>7036327526509</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>6248</t>
+          <t>6488</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2025-11-21T18:29:02-06:00</t>
+          <t>2025-11-27T20:04:51-06:00</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1302,12 +1302,12 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>BELEM LANDEROS PORRAS</t>
+          <t>ESTEBAN ORTIZ</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>BELEM LANDEROS PORRAS</t>
+          <t>ESTEBAN ORTIZ</t>
         </is>
       </c>
       <c r="H12" t="n">
@@ -1323,19 +1323,19 @@
         <v>2</v>
       </c>
       <c r="L12" t="n">
-        <v>18944.1</v>
+        <v>459</v>
       </c>
       <c r="M12" t="n">
-        <v>18944.11</v>
+        <v>459.01</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>20.9977224,-101.2963146</t>
+          <t>20.6498181,-100.3457546</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>20.9977224,-101.2963146</t>
+          <t>20.6498181,-100.3457546</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>SPRING_6248</t>
+          <t>SPRING_6488</t>
         </is>
       </c>
     </row>
@@ -1357,17 +1357,17 @@
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
-          <t>7017328279661</t>
+          <t>7036319301741</t>
         </is>
       </c>
       <c r="C13" s="1" t="inlineStr">
         <is>
-          <t>6247</t>
+          <t>6487</t>
         </is>
       </c>
       <c r="D13" s="1" t="inlineStr">
         <is>
-          <t>2025-11-21T17:47:53-06:00</t>
+          <t>2025-11-27T20:02:49-06:00</t>
         </is>
       </c>
       <c r="E13" s="1" t="inlineStr">
@@ -1377,40 +1377,40 @@
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>SAUL MONTERO HUICHAPEÑO</t>
+          <t>MIGUEL MENDOZA</t>
         </is>
       </c>
       <c r="G13" s="1" t="inlineStr">
         <is>
-          <t>SAUL MONTERO HUICHAPEÑO</t>
+          <t>MIGUEL MENDOZA</t>
         </is>
       </c>
       <c r="H13" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I13" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J13" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K13" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L13" s="1" t="n">
-        <v>4449</v>
+        <v>1648</v>
       </c>
       <c r="M13" s="1" t="n">
-        <v>4449.01</v>
+        <v>1648.01</v>
       </c>
       <c r="N13" s="1" t="inlineStr">
         <is>
-          <t>20.4863375,-100.9348244</t>
+          <t>19.3923495,-99.0709315</t>
         </is>
       </c>
       <c r="O13" s="1" t="inlineStr">
         <is>
-          <t>20.4863375,-100.9348244</t>
+          <t>19.3923495,-99.0709315</t>
         </is>
       </c>
       <c r="P13" s="1" t="inlineStr">
@@ -1420,7 +1420,7 @@
       </c>
       <c r="Q13" s="1" t="inlineStr">
         <is>
-          <t>SPRING_6247</t>
+          <t>SPRING_6487</t>
         </is>
       </c>
     </row>
@@ -1432,17 +1432,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>7017292398701</t>
+          <t>7036296101997</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>6246</t>
+          <t>6486</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2025-11-21T17:24:26-06:00</t>
+          <t>2025-11-27T19:53:51-06:00</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1452,12 +1452,12 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>LUIS MOSQUEDA</t>
+          <t>DARIANA DALILA VALENCIA RODRIGUEZ</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>LUIS MOSQUEDA</t>
+          <t>DARIANA DALILA VALENCIA RODRIGUEZ</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -1473,19 +1473,19 @@
         <v>2</v>
       </c>
       <c r="L14" t="n">
-        <v>5499</v>
+        <v>6497.05</v>
       </c>
       <c r="M14" t="n">
-        <v>5499.01</v>
+        <v>6497.06</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>20.3891657,-101.1835527</t>
+          <t>20.6556248,-103.2854636</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>20.3891657,-101.1835527</t>
+          <t>20.6556248,-103.2854636</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -1495,7 +1495,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>SPRING_6246</t>
+          <t>SPRING_6486</t>
         </is>
       </c>
     </row>
@@ -1507,17 +1507,17 @@
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
-          <t>7017203630189</t>
+          <t>7036147335277</t>
         </is>
       </c>
       <c r="C15" s="1" t="inlineStr">
         <is>
-          <t>6245</t>
+          <t>6485</t>
         </is>
       </c>
       <c r="D15" s="1" t="inlineStr">
         <is>
-          <t>2025-11-21T16:48:18-06:00</t>
+          <t>2025-11-27T19:05:04-06:00</t>
         </is>
       </c>
       <c r="E15" s="1" t="inlineStr">
@@ -1527,12 +1527,12 @@
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>MAURICIO NARANJO ZARZA</t>
+          <t>GIOVANNI ENRIQUE ELIGIO ATENO</t>
         </is>
       </c>
       <c r="G15" s="1" t="inlineStr">
         <is>
-          <t>MAURICIO NARANJO ZARZA</t>
+          <t>GIOVANNI ENRIQUE ELIGIO ATENO</t>
         </is>
       </c>
       <c r="H15" s="1" t="n">
@@ -1548,19 +1548,19 @@
         <v>2</v>
       </c>
       <c r="L15" s="1" t="n">
-        <v>5499</v>
+        <v>4449</v>
       </c>
       <c r="M15" s="1" t="n">
-        <v>5499.01</v>
+        <v>4449.01</v>
       </c>
       <c r="N15" s="1" t="inlineStr">
         <is>
-          <t>19.3689623,-99.2234549</t>
+          <t>20.0731763,-97.03514620000001</t>
         </is>
       </c>
       <c r="O15" s="1" t="inlineStr">
         <is>
-          <t>19.3689623,-99.2234549</t>
+          <t>20.0731763,-97.03514620000001</t>
         </is>
       </c>
       <c r="P15" s="1" t="inlineStr">
@@ -1570,7 +1570,7 @@
       </c>
       <c r="Q15" s="1" t="inlineStr">
         <is>
-          <t>SPRING_6245</t>
+          <t>SPRING_6485</t>
         </is>
       </c>
     </row>
@@ -1582,17 +1582,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>7017128755309</t>
+          <t>7036119810157</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>6244</t>
+          <t>6484</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2025-11-21T16:10:59-06:00</t>
+          <t>2025-11-27T18:55:30-06:00</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1602,40 +1602,40 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>SERGIO EDUARDO FERNANDEZ VEGA</t>
+          <t>GONZALO SANABRIA L</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>SERGIO EDUARDO FERNANDEZ VEGA</t>
+          <t>GONZALO SANABRIA L</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J16" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K16" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L16" t="n">
-        <v>18077.4</v>
+        <v>7149</v>
       </c>
       <c r="M16" t="n">
-        <v>18077.41</v>
+        <v>7149.01</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>19.2628276,-99.6353386</t>
+          <t>19.3217092,-99.0486605</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>19.2628276,-99.6353386</t>
+          <t>19.3217092,-99.0486605</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -1645,7 +1645,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>SPRING_6244</t>
+          <t>SPRING_6484</t>
         </is>
       </c>
     </row>
@@ -1657,17 +1657,17 @@
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>7017018163309</t>
+          <t>7036091859053</t>
         </is>
       </c>
       <c r="C17" s="1" t="inlineStr">
         <is>
-          <t>6243</t>
+          <t>6483</t>
         </is>
       </c>
       <c r="D17" s="1" t="inlineStr">
         <is>
-          <t>2025-11-21T15:18:51-06:00</t>
+          <t>2025-11-27T18:40:46-06:00</t>
         </is>
       </c>
       <c r="E17" s="1" t="inlineStr">
@@ -1677,40 +1677,40 @@
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>ALAN SALVADOR CAMACHO SANCHEZ</t>
+          <t>FELIPE SPINOLA</t>
         </is>
       </c>
       <c r="G17" s="1" t="inlineStr">
         <is>
-          <t>ALAN SALVADOR CAMACHO SANCHEZ</t>
+          <t>FELIPE SPINOLA</t>
         </is>
       </c>
       <c r="H17" s="1" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I17" s="1" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J17" s="1" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K17" s="1" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L17" s="1" t="n">
-        <v>7456.55</v>
+        <v>6409.65</v>
       </c>
       <c r="M17" s="1" t="n">
-        <v>7456.56</v>
+        <v>6409.66</v>
       </c>
       <c r="N17" s="1" t="inlineStr">
         <is>
-          <t>25.7697201,-109.012618</t>
+          <t>19.5070941,-99.2488173</t>
         </is>
       </c>
       <c r="O17" s="1" t="inlineStr">
         <is>
-          <t>25.7697201,-109.012618</t>
+          <t>19.5070941,-99.2488173</t>
         </is>
       </c>
       <c r="P17" s="1" t="inlineStr">
@@ -1720,7 +1720,7 @@
       </c>
       <c r="Q17" s="1" t="inlineStr">
         <is>
-          <t>SPRING_6243</t>
+          <t>SPRING_6483</t>
         </is>
       </c>
     </row>
@@ -1732,17 +1732,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>7016974385261</t>
+          <t>7036089532525</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>6242</t>
+          <t>6482</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2025-11-21T15:04:47-06:00</t>
+          <t>2025-11-27T18:39:20-06:00</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1752,12 +1752,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>RAUL FRAJA</t>
+          <t>JESÚS ALEJANDRO SOSA CORONA</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>RAUL FRAJA</t>
+          <t>JESÚS ALEJANDRO SOSA CORONA</t>
         </is>
       </c>
       <c r="H18" t="n">
@@ -1773,19 +1773,19 @@
         <v>2</v>
       </c>
       <c r="L18" t="n">
-        <v>4549</v>
+        <v>5499</v>
       </c>
       <c r="M18" t="n">
-        <v>4549.01</v>
+        <v>5499.01</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>19.4436122,-99.1762832</t>
+          <t>19.2826695,-99.6917492</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>19.4436122,-99.1762832</t>
+          <t>19.2826695,-99.6917492</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -1795,7 +1795,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>SPRING_6242</t>
+          <t>SPRING_6482</t>
         </is>
       </c>
     </row>
@@ -1807,17 +1807,17 @@
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t>7016938438765</t>
+          <t>7036053848173</t>
         </is>
       </c>
       <c r="C19" s="1" t="inlineStr">
         <is>
-          <t>6241</t>
+          <t>6481</t>
         </is>
       </c>
       <c r="D19" s="1" t="inlineStr">
         <is>
-          <t>2025-11-21T14:47:20-06:00</t>
+          <t>2025-11-27T18:22:51-06:00</t>
         </is>
       </c>
       <c r="E19" s="1" t="inlineStr">
@@ -1827,12 +1827,12 @@
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>JOAQUIN PEREZ VALERA</t>
+          <t>AURELIANO MANCERA BEDOLLA</t>
         </is>
       </c>
       <c r="G19" s="1" t="inlineStr">
         <is>
-          <t>JOAQUIN PEREZ VALERA</t>
+          <t>AURELIANO MANCERA BEDOLLA</t>
         </is>
       </c>
       <c r="H19" s="1" t="n">
@@ -1848,19 +1848,19 @@
         <v>2</v>
       </c>
       <c r="L19" s="1" t="n">
-        <v>5399</v>
+        <v>18944.1</v>
       </c>
       <c r="M19" s="1" t="n">
-        <v>5399.01</v>
+        <v>18944.11</v>
       </c>
       <c r="N19" s="1" t="inlineStr">
         <is>
-          <t>20.8660559,-103.4342002</t>
+          <t>19.4842805,-99.2316037</t>
         </is>
       </c>
       <c r="O19" s="1" t="inlineStr">
         <is>
-          <t>20.8660559,-103.4342002</t>
+          <t>19.4842805,-99.2316037</t>
         </is>
       </c>
       <c r="P19" s="1" t="inlineStr">
@@ -1870,7 +1870,7 @@
       </c>
       <c r="Q19" s="1" t="inlineStr">
         <is>
-          <t>SPRING_6241</t>
+          <t>SPRING_6481</t>
         </is>
       </c>
     </row>
@@ -1882,17 +1882,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>7016823226477</t>
+          <t>7036047556717</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>6240</t>
+          <t>6480</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2025-11-21T13:59:42-06:00</t>
+          <t>2025-11-27T18:21:08-06:00</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1902,12 +1902,12 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>DULCE CAMPOS</t>
+          <t>FELIPE SPINOLA</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>DULCE CAMPOS</t>
+          <t>FELIPE SPINOLA</t>
         </is>
       </c>
       <c r="H20" t="n">
@@ -1923,19 +1923,19 @@
         <v>2</v>
       </c>
       <c r="L20" t="n">
-        <v>7149</v>
+        <v>5749</v>
       </c>
       <c r="M20" t="n">
-        <v>7149.01</v>
+        <v>5749.01</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>19.7148213,-99.22490490000001</t>
+          <t>19.5070941,-99.2488173</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>19.7148213,-99.22490490000001</t>
+          <t>19.5070941,-99.2488173</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -1945,7 +1945,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>SPRING_6240</t>
+          <t>SPRING_6480</t>
         </is>
       </c>
     </row>
@@ -1957,17 +1957,17 @@
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t>7016819621997</t>
+          <t>7035961671789</t>
         </is>
       </c>
       <c r="C21" s="1" t="inlineStr">
         <is>
-          <t>6239</t>
+          <t>6479</t>
         </is>
       </c>
       <c r="D21" s="1" t="inlineStr">
         <is>
-          <t>2025-11-21T13:57:36-06:00</t>
+          <t>2025-11-27T17:51:35-06:00</t>
         </is>
       </c>
       <c r="E21" s="1" t="inlineStr">
@@ -1977,36 +1977,50 @@
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>CLAUDIA LIZETH FONSECA FLORES</t>
-        </is>
-      </c>
-      <c r="G21" s="1" t="inlineStr"/>
+          <t>IVETTE BRUCIAGA OJEDA</t>
+        </is>
+      </c>
+      <c r="G21" s="1" t="inlineStr">
+        <is>
+          <t>IVETTE BRUCIAGA OJEDA</t>
+        </is>
+      </c>
       <c r="H21" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="I21" s="1" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="I21" s="1" t="n">
+        <v>2</v>
+      </c>
       <c r="J21" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="K21" s="1" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="K21" s="1" t="n">
+        <v>2</v>
+      </c>
       <c r="L21" s="1" t="n">
-        <v>5048</v>
-      </c>
-      <c r="M21" s="1" t="inlineStr"/>
+        <v>37889.1</v>
+      </c>
+      <c r="M21" s="1" t="n">
+        <v>37889.11</v>
+      </c>
       <c r="N21" s="1" t="inlineStr">
         <is>
-          <t>21.5330917,-104.9128183</t>
-        </is>
-      </c>
-      <c r="O21" s="1" t="inlineStr"/>
+          <t>24.0348441,-104.6274569</t>
+        </is>
+      </c>
+      <c r="O21" s="1" t="inlineStr">
+        <is>
+          <t>24.0348441,-104.6274569</t>
+        </is>
+      </c>
       <c r="P21" s="1" t="inlineStr">
         <is>
-          <t>NO ENCONTRADO EN INTELISIS</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="Q21" s="1" t="inlineStr">
         <is>
-          <t>SPRING_6239</t>
+          <t>SPRING_6479</t>
         </is>
       </c>
     </row>
@@ -2018,17 +2032,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>7016697725037</t>
+          <t>7035945353325</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>6238</t>
+          <t>6478</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2025-11-21T13:04:53-06:00</t>
+          <t>2025-11-27T17:42:00-06:00</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2038,50 +2052,50 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>MARÍA DE LA LUZ RIVERA RIVERA</t>
+          <t>DANIEL RAMOS</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>MARÍA DE LA LUZ RIVERA RIVERA</t>
+          <t>DANIEL RAMOS</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L22" t="n">
-        <v>10119.08</v>
+        <v>16068</v>
       </c>
       <c r="M22" t="n">
-        <v>10119.08</v>
+        <v>16068.01</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>18.1387806,-93.00631349999999</t>
+          <t>19.1131412,-104.3328967</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>18.1387806,-93.00631349999999</t>
+          <t>19.1131412,-104.3328967</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>Cantidad dif (1.0 vs 2.0) | Registros dif (1 vs 2)</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>SPRING_6238</t>
+          <t>SPRING_6478</t>
         </is>
       </c>
     </row>
@@ -2093,17 +2107,17 @@
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
-          <t>7016677965933</t>
+          <t>7035941585005</t>
         </is>
       </c>
       <c r="C23" s="1" t="inlineStr">
         <is>
-          <t>6237</t>
+          <t>6477</t>
         </is>
       </c>
       <c r="D23" s="1" t="inlineStr">
         <is>
-          <t>2025-11-21T12:58:16-06:00</t>
+          <t>2025-11-27T17:39:46-06:00</t>
         </is>
       </c>
       <c r="E23" s="1" t="inlineStr">
@@ -2113,12 +2127,12 @@
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>MARTHA ANDREA NERIA LOPEZ</t>
+          <t>IVONNE GARCIA</t>
         </is>
       </c>
       <c r="G23" s="1" t="inlineStr">
         <is>
-          <t>MARTHA ANDREA NERIA LOPEZ</t>
+          <t>IVONNE GARCIA</t>
         </is>
       </c>
       <c r="H23" s="1" t="n">
@@ -2134,19 +2148,19 @@
         <v>2</v>
       </c>
       <c r="L23" s="1" t="n">
-        <v>349</v>
+        <v>749</v>
       </c>
       <c r="M23" s="1" t="n">
-        <v>349.01</v>
+        <v>749.01</v>
       </c>
       <c r="N23" s="1" t="inlineStr">
         <is>
-          <t>19.3572178,-99.11638350000001</t>
+          <t>19.3626432,-98.9974162</t>
         </is>
       </c>
       <c r="O23" s="1" t="inlineStr">
         <is>
-          <t>19.3572178,-99.11638350000001</t>
+          <t>19.3626432,-98.9974162</t>
         </is>
       </c>
       <c r="P23" s="1" t="inlineStr">
@@ -2156,7 +2170,7 @@
       </c>
       <c r="Q23" s="1" t="inlineStr">
         <is>
-          <t>SPRING_6237</t>
+          <t>SPRING_6477</t>
         </is>
       </c>
     </row>
@@ -2168,17 +2182,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>7016640217197</t>
+          <t>7035803893869</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>6236</t>
+          <t>6476</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2025-11-21T12:38:11-06:00</t>
+          <t>2025-11-27T16:45:41-06:00</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2188,40 +2202,40 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>DANIEL ZOZAYA VALDES</t>
+          <t>CELINA HERRERA GONZÁLEZ</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>DANIEL ZOZAYA VALDES</t>
+          <t>CELINA HERRERA GONZÁLEZ</t>
         </is>
       </c>
       <c r="H24" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I24" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J24" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K24" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L24" t="n">
-        <v>21741.3</v>
+        <v>4799</v>
       </c>
       <c r="M24" t="n">
-        <v>21741.31</v>
+        <v>4799</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>19.4110451,-99.1654829</t>
+          <t>25.738819,-100.2906632</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>19.4110451,-99.1654829</t>
+          <t>25.738819,-100.2906632</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -2231,7 +2245,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>SPRING_6236</t>
+          <t>SPRING_6476</t>
         </is>
       </c>
     </row>
@@ -2243,17 +2257,17 @@
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
-          <t>7016552267885</t>
+          <t>7035803238509</t>
         </is>
       </c>
       <c r="C25" s="1" t="inlineStr">
         <is>
-          <t>6235</t>
+          <t>6475</t>
         </is>
       </c>
       <c r="D25" s="1" t="inlineStr">
         <is>
-          <t>2025-11-21T12:06:03-06:00</t>
+          <t>2025-11-27T16:45:20-06:00</t>
         </is>
       </c>
       <c r="E25" s="1" t="inlineStr">
@@ -2263,12 +2277,12 @@
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>CINDY LARA</t>
+          <t>SELINE MOTA</t>
         </is>
       </c>
       <c r="G25" s="1" t="inlineStr">
         <is>
-          <t>CINDY LARA</t>
+          <t>SELINE MOTA</t>
         </is>
       </c>
       <c r="H25" s="1" t="n">
@@ -2284,19 +2298,19 @@
         <v>2</v>
       </c>
       <c r="L25" s="1" t="n">
-        <v>4549</v>
+        <v>6099</v>
       </c>
       <c r="M25" s="1" t="n">
-        <v>4549.01</v>
+        <v>6099.01</v>
       </c>
       <c r="N25" s="1" t="inlineStr">
         <is>
-          <t>19.524732,-99.193388</t>
+          <t>19.3540967,-99.1898653</t>
         </is>
       </c>
       <c r="O25" s="1" t="inlineStr">
         <is>
-          <t>19.524732,-99.193388</t>
+          <t>19.3540967,-99.1898653</t>
         </is>
       </c>
       <c r="P25" s="1" t="inlineStr">
@@ -2306,7 +2320,7 @@
       </c>
       <c r="Q25" s="1" t="inlineStr">
         <is>
-          <t>SPRING_6235</t>
+          <t>SPRING_6475</t>
         </is>
       </c>
     </row>
@@ -2318,17 +2332,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>7016466481261</t>
+          <t>7035790393453</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>6234</t>
+          <t>6474</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2025-11-21T11:28:40-06:00</t>
+          <t>2025-11-27T16:35:21-06:00</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2338,12 +2352,12 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>CÉSAR IAN CANTORAL OLAN</t>
+          <t>HUMBERTO NAVARRO</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>CÉSAR IAN CANTORAL OLAN</t>
+          <t>HUMBERTO NAVARRO</t>
         </is>
       </c>
       <c r="H26" t="n">
@@ -2359,19 +2373,19 @@
         <v>2</v>
       </c>
       <c r="L26" t="n">
-        <v>6249</v>
+        <v>4449</v>
       </c>
       <c r="M26" t="n">
-        <v>6249.01</v>
+        <v>4449.01</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>18.172667,-93.06450670000001</t>
+          <t>19.7016854,-103.4802218</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>18.172667,-93.06450670000001</t>
+          <t>19.7016854,-103.4802218</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -2381,7 +2395,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>SPRING_6234</t>
+          <t>SPRING_6474</t>
         </is>
       </c>
     </row>
@@ -2393,17 +2407,17 @@
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
-          <t>7016350941293</t>
+          <t>7035783348333</t>
         </is>
       </c>
       <c r="C27" s="1" t="inlineStr">
         <is>
-          <t>6233</t>
+          <t>6473</t>
         </is>
       </c>
       <c r="D27" s="1" t="inlineStr">
         <is>
-          <t>2025-11-21T10:56:27-06:00</t>
+          <t>2025-11-27T16:30:15-06:00</t>
         </is>
       </c>
       <c r="E27" s="1" t="inlineStr">
@@ -2413,12 +2427,12 @@
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>SANTIAGO CÉSAR GARZA PÉREZ</t>
+          <t>ALEXIS CALVARIO HERNANDEZ</t>
         </is>
       </c>
       <c r="G27" s="1" t="inlineStr">
         <is>
-          <t>SANTIAGO CÉSAR GARZA PÉREZ</t>
+          <t>ALEXIS CALVARIO HERNANDEZ</t>
         </is>
       </c>
       <c r="H27" s="1" t="n">
@@ -2434,19 +2448,19 @@
         <v>2</v>
       </c>
       <c r="L27" s="1" t="n">
-        <v>4749</v>
+        <v>12584.68</v>
       </c>
       <c r="M27" s="1" t="n">
-        <v>4749.01</v>
+        <v>12584.69</v>
       </c>
       <c r="N27" s="1" t="inlineStr">
         <is>
-          <t>18.9708977,-99.138121</t>
+          <t>19.3569024,-99.21898379999999</t>
         </is>
       </c>
       <c r="O27" s="1" t="inlineStr">
         <is>
-          <t>18.9708977,-99.138121</t>
+          <t>19.3569024,-99.21898379999999</t>
         </is>
       </c>
       <c r="P27" s="1" t="inlineStr">
@@ -2456,7 +2470,7 @@
       </c>
       <c r="Q27" s="1" t="inlineStr">
         <is>
-          <t>SPRING_6233</t>
+          <t>SPRING_6473</t>
         </is>
       </c>
     </row>
@@ -2468,17 +2482,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>7016302542957</t>
+          <t>7035781185645</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>6232</t>
+          <t>6472</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2025-11-21T10:31:35-06:00</t>
+          <t>2025-11-27T16:28:51-06:00</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2488,50 +2502,36 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>OBED LACHICA GARCIA</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>OBED LACHICA GARCIA</t>
-        </is>
-      </c>
+          <t>ANGEL GRANADOS</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>3</v>
-      </c>
-      <c r="I28" t="n">
-        <v>3</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="I28" t="inlineStr"/>
       <c r="J28" t="n">
         <v>3</v>
       </c>
-      <c r="K28" t="n">
-        <v>3</v>
-      </c>
+      <c r="K28" t="inlineStr"/>
       <c r="L28" t="n">
-        <v>16068</v>
-      </c>
-      <c r="M28" t="n">
-        <v>16068.01</v>
-      </c>
+        <v>26576</v>
+      </c>
+      <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr">
         <is>
-          <t>28.6332216,-106.0604036</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>28.6332216,-106.0604036</t>
-        </is>
-      </c>
+          <t>20.5415158,-100.4461882</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>NO ENCONTRADO EN INTELISIS</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>SPRING_6232</t>
+          <t>SPRING_6472</t>
         </is>
       </c>
     </row>
@@ -2543,17 +2543,17 @@
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
-          <t>7016252178541</t>
+          <t>7035618394221</t>
         </is>
       </c>
       <c r="C29" s="1" t="inlineStr">
         <is>
-          <t>6231</t>
+          <t>6471</t>
         </is>
       </c>
       <c r="D29" s="1" t="inlineStr">
         <is>
-          <t>2025-11-21T10:13:01-06:00</t>
+          <t>2025-11-27T15:08:44-06:00</t>
         </is>
       </c>
       <c r="E29" s="1" t="inlineStr">
@@ -2563,12 +2563,12 @@
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>DULCE TOVAR GALICIA</t>
+          <t>SAMAHI LEYVA MARTÍNEZ</t>
         </is>
       </c>
       <c r="G29" s="1" t="inlineStr">
         <is>
-          <t>DULCE TOVAR GALICIA</t>
+          <t>SAMAHI LEYVA MARTÍNEZ</t>
         </is>
       </c>
       <c r="H29" s="1" t="n">
@@ -2584,19 +2584,19 @@
         <v>3</v>
       </c>
       <c r="L29" s="1" t="n">
-        <v>1208</v>
+        <v>1598</v>
       </c>
       <c r="M29" s="1" t="n">
-        <v>1208.01</v>
+        <v>1598.01</v>
       </c>
       <c r="N29" s="1" t="inlineStr">
         <is>
-          <t>19.3777695,-99.19762419999999</t>
+          <t>17.0829992,-96.7514124</t>
         </is>
       </c>
       <c r="O29" s="1" t="inlineStr">
         <is>
-          <t>19.3777695,-99.19762419999999</t>
+          <t>17.0829992,-96.7514124</t>
         </is>
       </c>
       <c r="P29" s="1" t="inlineStr">
@@ -2606,7 +2606,7 @@
       </c>
       <c r="Q29" s="1" t="inlineStr">
         <is>
-          <t>SPRING_6231</t>
+          <t>SPRING_6471</t>
         </is>
       </c>
     </row>
@@ -2618,17 +2618,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>7016180777069</t>
+          <t>7035550531693</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>6230</t>
+          <t>6470</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2025-11-21T09:43:51-06:00</t>
+          <t>2025-11-27T14:26:05-06:00</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2638,40 +2638,40 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>MANUEL G ALONSO ESPINOSA</t>
+          <t>VICTOR GONZALEZ  BARRIENTOS</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>MANUEL G ALONSO ESPINOSA</t>
+          <t>VICTOR GONZALEZ  BARRIENTOS</t>
         </is>
       </c>
       <c r="H30" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="I30" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J30" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K30" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L30" t="n">
-        <v>41931.9</v>
+        <v>5749</v>
       </c>
       <c r="M30" t="n">
-        <v>41931.91</v>
+        <v>5749.01</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>21.0109283,-88.3075762</t>
+          <t>19.4019743,-99.0084341</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>21.0109283,-88.3075762</t>
+          <t>19.4019743,-99.0084341</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -2681,7 +2681,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>SPRING_6230</t>
+          <t>SPRING_6470</t>
         </is>
       </c>
     </row>
@@ -2693,17 +2693,17 @@
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
-          <t>7015365443693</t>
+          <t>7035511275629</t>
         </is>
       </c>
       <c r="C31" s="1" t="inlineStr">
         <is>
-          <t>6228</t>
+          <t>6469</t>
         </is>
       </c>
       <c r="D31" s="1" t="inlineStr">
         <is>
-          <t>2025-11-21T03:13:33-06:00</t>
+          <t>2025-11-27T14:10:32-06:00</t>
         </is>
       </c>
       <c r="E31" s="1" t="inlineStr">
@@ -2713,12 +2713,12 @@
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>JONATHAN FROYLAN COLIN ALVARADO</t>
+          <t>CARMEN GARCIA</t>
         </is>
       </c>
       <c r="G31" s="1" t="inlineStr">
         <is>
-          <t>JONATHAN FROYLAN COLIN ALVARADO</t>
+          <t>CARMEN GARCIA</t>
         </is>
       </c>
       <c r="H31" s="1" t="n">
@@ -2734,19 +2734,19 @@
         <v>2</v>
       </c>
       <c r="L31" s="1" t="n">
-        <v>7199</v>
+        <v>18944.1</v>
       </c>
       <c r="M31" s="1" t="n">
-        <v>7199.01</v>
+        <v>18944.11</v>
       </c>
       <c r="N31" s="1" t="inlineStr">
         <is>
-          <t>20.4436657,-103.2636529</t>
+          <t>19.6208273,-99.2548599</t>
         </is>
       </c>
       <c r="O31" s="1" t="inlineStr">
         <is>
-          <t>20.4436657,-103.2636529</t>
+          <t>19.6208273,-99.2548599</t>
         </is>
       </c>
       <c r="P31" s="1" t="inlineStr">
@@ -2756,7 +2756,7 @@
       </c>
       <c r="Q31" s="1" t="inlineStr">
         <is>
-          <t>SPRING_6228</t>
+          <t>SPRING_6469</t>
         </is>
       </c>
     </row>
@@ -2768,17 +2768,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>7014726631533</t>
+          <t>7035468939373</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>6227</t>
+          <t>6468</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2025-11-21T00:01:47-06:00</t>
+          <t>2025-11-27T13:50:13-06:00</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2788,40 +2788,40 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>CARLOS EDUARDO GOMEZ CUARENTA</t>
+          <t>GARCÍA GUILLÉN INGRID MONTSERRAT</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>CARLOS EDUARDO GOMEZ CUARENTA</t>
+          <t>GARCÍA GUILLÉN INGRID MONTSERRAT</t>
         </is>
       </c>
       <c r="H32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L32" t="n">
-        <v>10265.36</v>
+        <v>899</v>
       </c>
       <c r="M32" t="n">
-        <v>10265.37</v>
+        <v>899.01</v>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>20.5192237,-103.2403779</t>
+          <t>19.6831837,-99.2042925</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>20.5192237,-103.2403779</t>
+          <t>19.6831837,-99.2042925</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
@@ -2831,29 +2831,29 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>SPRING_6227</t>
+          <t>SPRING_6468</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>ATLAS</t>
+          <t>SPRING</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
-          <t>6093685096501</t>
+          <t>7035451179117</t>
         </is>
       </c>
       <c r="C33" s="1" t="inlineStr">
         <is>
-          <t>18863</t>
+          <t>6467</t>
         </is>
       </c>
       <c r="D33" s="1" t="inlineStr">
         <is>
-          <t>2025-11-21T23:03:35-06:00</t>
+          <t>2025-11-27T13:36:52-06:00</t>
         </is>
       </c>
       <c r="E33" s="1" t="inlineStr">
@@ -2863,40 +2863,40 @@
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>FRANCISCO ALTAMIRA RIVERA</t>
+          <t>DIANA PAOLA GUZMAN</t>
         </is>
       </c>
       <c r="G33" s="1" t="inlineStr">
         <is>
-          <t>FRANCISCO ALTAMIRA RIVERA</t>
+          <t>DIANA PAOLA GUZMAN</t>
         </is>
       </c>
       <c r="H33" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I33" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J33" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K33" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L33" s="1" t="n">
-        <v>2499</v>
+        <v>4449</v>
       </c>
       <c r="M33" s="1" t="n">
-        <v>2499</v>
+        <v>4449.01</v>
       </c>
       <c r="N33" s="1" t="inlineStr">
         <is>
-          <t>19.1499988,-96.9679199</t>
+          <t>19.9460665,-96.8538288</t>
         </is>
       </c>
       <c r="O33" s="1" t="inlineStr">
         <is>
-          <t>19.1499988,-96.9679199</t>
+          <t>19.9460665,-96.8538288</t>
         </is>
       </c>
       <c r="P33" s="1" t="inlineStr">
@@ -2906,29 +2906,29 @@
       </c>
       <c r="Q33" s="1" t="inlineStr">
         <is>
-          <t>ATLAS_18863</t>
+          <t>SPRING_6467</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ATLAS</t>
+          <t>SPRING</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>6093665534005</t>
+          <t>7035356184685</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>18862</t>
+          <t>6466</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2025-11-21T22:43:50-06:00</t>
+          <t>2025-11-27T12:52:06-06:00</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2938,12 +2938,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>ABRIL SAC NICTE CATZIM ESPINOSA</t>
+          <t>ANGEL DE JESÚS HERNÁNDEZ BASILIO</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>ABRIL SAC NICTE CATZIM ESPINOSA</t>
+          <t>ANGEL DE JESÚS HERNÁNDEZ BASILIO</t>
         </is>
       </c>
       <c r="H34" t="n">
@@ -2959,19 +2959,19 @@
         <v>2</v>
       </c>
       <c r="L34" t="n">
-        <v>6998</v>
+        <v>3899</v>
       </c>
       <c r="M34" t="n">
-        <v>6998</v>
+        <v>3899.01</v>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>18.1445756,-92.8557999</t>
+          <t>17.0579962,-96.69923670000001</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>18.1445756,-92.8557999</t>
+          <t>17.0579962,-96.69923670000001</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
@@ -2981,29 +2981,29 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>ATLAS_18862</t>
+          <t>SPRING_6466</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>ATLAS</t>
+          <t>SPRING</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
-          <t>6093576241205</t>
+          <t>7035333967981</t>
         </is>
       </c>
       <c r="C35" s="1" t="inlineStr">
         <is>
-          <t>18861</t>
+          <t>6465</t>
         </is>
       </c>
       <c r="D35" s="1" t="inlineStr">
         <is>
-          <t>2025-11-21T21:16:10-06:00</t>
+          <t>2025-11-27T12:38:10-06:00</t>
         </is>
       </c>
       <c r="E35" s="1" t="inlineStr">
@@ -3013,72 +3013,72 @@
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>LIBRADO MENDEZ</t>
+          <t>MA. DEL CARMEN VÁZQUEZ MARTINEZ</t>
         </is>
       </c>
       <c r="G35" s="1" t="inlineStr">
         <is>
-          <t>LIBRADO MENDEZ</t>
+          <t>MA. DEL CARMEN VÁZQUEZ MARTINEZ</t>
         </is>
       </c>
       <c r="H35" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I35" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J35" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K35" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L35" s="1" t="n">
-        <v>1358</v>
+        <v>9398</v>
       </c>
       <c r="M35" s="1" t="n">
-        <v>1358</v>
+        <v>9398.01</v>
       </c>
       <c r="N35" s="1" t="inlineStr">
         <is>
-          <t>14.8924915,-92.25142269999999</t>
+          <t>18.9159617,-99.2448007</t>
         </is>
       </c>
       <c r="O35" s="1" t="inlineStr">
         <is>
-          <t>14.8924915,-92.25142269999999</t>
+          <t>18.9159617,-99.2448007</t>
         </is>
       </c>
       <c r="P35" s="1" t="inlineStr">
         <is>
-          <t>Cantidad dif (1.0 vs 2.0) | Registros dif (1 vs 2)</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="Q35" s="1" t="inlineStr">
         <is>
-          <t>ATLAS_18861</t>
+          <t>SPRING_6465</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ATLAS</t>
+          <t>SPRING</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>6092917702709</t>
+          <t>7035328692333</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>18860</t>
+          <t>6464</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2025-11-21T14:42:18-06:00</t>
+          <t>2025-11-27T12:34:37-06:00</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3088,58 +3088,72 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>PABLO BALTAZAR MONTÚFAR</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr"/>
+          <t>LUIS ANGEL SERVIN FUENTES</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>LUIS ANGEL SERVIN FUENTES</t>
+        </is>
+      </c>
       <c r="H36" t="n">
-        <v>1</v>
-      </c>
-      <c r="I36" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="I36" t="n">
+        <v>2</v>
+      </c>
       <c r="J36" t="n">
-        <v>1</v>
-      </c>
-      <c r="K36" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="K36" t="n">
+        <v>2</v>
+      </c>
       <c r="L36" t="n">
-        <v>8519</v>
-      </c>
-      <c r="M36" t="inlineStr"/>
+        <v>9686.68</v>
+      </c>
+      <c r="M36" t="n">
+        <v>9686.690000000001</v>
+      </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>19.2797542,-99.1642376</t>
-        </is>
-      </c>
-      <c r="O36" t="inlineStr"/>
+          <t>16.1866799,-95.200316</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>16.1866799,-95.200316</t>
+        </is>
+      </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>NO ENCONTRADO EN INTELISIS</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>ATLAS_18860</t>
+          <t>SPRING_6464</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>ATLAS</t>
+          <t>SPRING</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
-          <t>6092826935349</t>
+          <t>7035169341549</t>
         </is>
       </c>
       <c r="C37" s="1" t="inlineStr">
         <is>
-          <t>18859</t>
+          <t>6463</t>
         </is>
       </c>
       <c r="D37" s="1" t="inlineStr">
         <is>
-          <t>2025-11-21T13:53:14-06:00</t>
+          <t>2025-11-27T11:18:16-06:00</t>
         </is>
       </c>
       <c r="E37" s="1" t="inlineStr">
@@ -3149,40 +3163,40 @@
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>PEDRO ROBERTO QUINTERO CANTU</t>
+          <t>OSCAR LOPEZ RUIZ</t>
         </is>
       </c>
       <c r="G37" s="1" t="inlineStr">
         <is>
-          <t>PEDRO ROBERTO QUINTERO CANTU</t>
+          <t>OSCAR LOPEZ RUIZ</t>
         </is>
       </c>
       <c r="H37" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I37" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J37" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K37" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L37" s="1" t="n">
-        <v>9649</v>
+        <v>4549</v>
       </c>
       <c r="M37" s="1" t="n">
-        <v>9649</v>
+        <v>4549.01</v>
       </c>
       <c r="N37" s="1" t="inlineStr">
         <is>
-          <t>18.9046218,-99.17708929999999</t>
+          <t>17.9637192,-102.2229993</t>
         </is>
       </c>
       <c r="O37" s="1" t="inlineStr">
         <is>
-          <t>18.9046218,-99.17708929999999</t>
+          <t>17.9637192,-102.2229993</t>
         </is>
       </c>
       <c r="P37" s="1" t="inlineStr">
@@ -3192,29 +3206,29 @@
       </c>
       <c r="Q37" s="1" t="inlineStr">
         <is>
-          <t>ATLAS_18859</t>
+          <t>SPRING_6463</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ATLAS</t>
+          <t>SPRING</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>6092805308469</t>
+          <t>7035084243053</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>18858</t>
+          <t>6462</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2025-11-21T13:41:27-06:00</t>
+          <t>2025-11-27T10:41:46-06:00</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3224,58 +3238,72 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>MAURICIO RUEDA ANAYA</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr"/>
+          <t>JUAN ANTONIO ROJAS MARTINEZ</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>JUAN ANTONIO ROJAS MARTINEZ</t>
+        </is>
+      </c>
       <c r="H38" t="n">
-        <v>1</v>
-      </c>
-      <c r="I38" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="I38" t="n">
+        <v>4</v>
+      </c>
       <c r="J38" t="n">
-        <v>1</v>
-      </c>
-      <c r="K38" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="K38" t="n">
+        <v>2</v>
+      </c>
       <c r="L38" t="n">
-        <v>9919</v>
-      </c>
-      <c r="M38" t="inlineStr"/>
+        <v>2607</v>
+      </c>
+      <c r="M38" t="n">
+        <v>2607.01</v>
+      </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>19.3511098,-99.29539729999999</t>
-        </is>
-      </c>
-      <c r="O38" t="inlineStr"/>
+          <t>19.296073,-99.0443251</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>19.296073,-99.0443251</t>
+        </is>
+      </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>NO ENCONTRADO EN INTELISIS</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>ATLAS_18858</t>
+          <t>SPRING_6462</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>ATLAS</t>
+          <t>SPRING</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
-          <t>6092751175733</t>
+          <t>7034949927021</t>
         </is>
       </c>
       <c r="C39" s="1" t="inlineStr">
         <is>
-          <t>18857</t>
+          <t>6461</t>
         </is>
       </c>
       <c r="D39" s="1" t="inlineStr">
         <is>
-          <t>2025-11-21T13:15:28-06:00</t>
+          <t>2025-11-27T09:40:19-06:00</t>
         </is>
       </c>
       <c r="E39" s="1" t="inlineStr">
@@ -3285,40 +3313,40 @@
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>LUIS ENRIQUE MARTÍNEZ GARCÍA</t>
+          <t>CESAR CRUZ</t>
         </is>
       </c>
       <c r="G39" s="1" t="inlineStr">
         <is>
-          <t>LUIS ENRIQUE MARTÍNEZ GARCÍA</t>
+          <t>CESAR CRUZ</t>
         </is>
       </c>
       <c r="H39" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I39" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J39" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K39" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L39" s="1" t="n">
-        <v>8349</v>
+        <v>1738</v>
       </c>
       <c r="M39" s="1" t="n">
-        <v>8349</v>
+        <v>1738.01</v>
       </c>
       <c r="N39" s="1" t="inlineStr">
         <is>
-          <t>19.4580039,-99.1910114</t>
+          <t>19.3837511,-99.1659839</t>
         </is>
       </c>
       <c r="O39" s="1" t="inlineStr">
         <is>
-          <t>19.4580039,-99.1910114</t>
+          <t>19.3837511,-99.1659839</t>
         </is>
       </c>
       <c r="P39" s="1" t="inlineStr">
@@ -3328,29 +3356,29 @@
       </c>
       <c r="Q39" s="1" t="inlineStr">
         <is>
-          <t>ATLAS_18857</t>
+          <t>SPRING_6461</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ATLAS</t>
+          <t>SPRING</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>6092518981685</t>
+          <t>7034942619757</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>18856</t>
+          <t>6460</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2025-11-21T11:55:02-06:00</t>
+          <t>2025-11-27T09:35:34-06:00</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3360,40 +3388,40 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>EDUARDO DIAZ DIAZ</t>
+          <t>LAURA LILIA PIEDRAS CARRILLO</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>EDUARDO DIAZ DIAZ</t>
+          <t>LAURA LILIA PIEDRAS CARRILLO</t>
         </is>
       </c>
       <c r="H40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L40" t="n">
-        <v>9919</v>
+        <v>4549</v>
       </c>
       <c r="M40" t="n">
-        <v>9919</v>
+        <v>4549.01</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>19.2726201,-99.6828147</t>
+          <t>19.4188716,-98.8863491</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>19.2726201,-99.6828147</t>
+          <t>19.4188716,-98.8863491</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
@@ -3403,29 +3431,29 @@
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>ATLAS_18856</t>
+          <t>SPRING_6460</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>ATLAS</t>
+          <t>SPRING</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
-          <t>6092360613941</t>
+          <t>7034935738477</t>
         </is>
       </c>
       <c r="C41" s="1" t="inlineStr">
         <is>
-          <t>18855</t>
+          <t>6459</t>
         </is>
       </c>
       <c r="D41" s="1" t="inlineStr">
         <is>
-          <t>2025-11-21T11:14:36-06:00</t>
+          <t>2025-11-27T09:30:55-06:00</t>
         </is>
       </c>
       <c r="E41" s="1" t="inlineStr">
@@ -3435,125 +3463,1850 @@
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>NORBERTO GUEVARA TRABANCO</t>
+          <t>ABIGAIL GALLARDO MARTINEZ</t>
         </is>
       </c>
       <c r="G41" s="1" t="inlineStr">
         <is>
-          <t>NORBERTO GUEVARA TRABANCO</t>
+          <t>ABIGAIL GALLARDO MARTINEZ</t>
         </is>
       </c>
       <c r="H41" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I41" s="1" t="n">
         <v>2</v>
       </c>
       <c r="J41" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K41" s="1" t="n">
         <v>2</v>
       </c>
       <c r="L41" s="1" t="n">
-        <v>1098</v>
+        <v>23549</v>
       </c>
       <c r="M41" s="1" t="n">
-        <v>1098</v>
+        <v>23549.01</v>
       </c>
       <c r="N41" s="1" t="inlineStr">
         <is>
-          <t>19.2819346,-99.2034504</t>
+          <t>19.0513105,-98.2703588</t>
         </is>
       </c>
       <c r="O41" s="1" t="inlineStr">
         <is>
-          <t>19.2819346,-99.2034504</t>
+          <t>19.0513105,-98.2703588</t>
         </is>
       </c>
       <c r="P41" s="1" t="inlineStr">
         <is>
-          <t>Cantidad dif (1.0 vs 2.0) | Registros dif (1 vs 2)</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="Q41" s="1" t="inlineStr">
         <is>
-          <t>ATLAS_18855</t>
+          <t>SPRING_6459</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>SPRING</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>7034923155565</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>6458</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2025-11-27T09:23:19-06:00</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>DAVID OLIVAR ROJAS</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>DAVID OLIVAR ROJAS</t>
+        </is>
+      </c>
+      <c r="H42" t="n">
+        <v>5</v>
+      </c>
+      <c r="I42" t="n">
+        <v>5</v>
+      </c>
+      <c r="J42" t="n">
+        <v>3</v>
+      </c>
+      <c r="K42" t="n">
+        <v>3</v>
+      </c>
+      <c r="L42" t="n">
+        <v>15476.4</v>
+      </c>
+      <c r="M42" t="n">
+        <v>15476.41</v>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>18.6754408,-98.9550213</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>18.6754408,-98.9550213</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>SPRING_6458</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="inlineStr">
+        <is>
+          <t>SPRING</t>
+        </is>
+      </c>
+      <c r="B43" s="1" t="inlineStr">
+        <is>
+          <t>7034917847149</t>
+        </is>
+      </c>
+      <c r="C43" s="1" t="inlineStr">
+        <is>
+          <t>6457</t>
+        </is>
+      </c>
+      <c r="D43" s="1" t="inlineStr">
+        <is>
+          <t>2025-11-27T09:21:14-06:00</t>
+        </is>
+      </c>
+      <c r="E43" s="1" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="F43" s="1" t="inlineStr">
+        <is>
+          <t>ALBERTO LARA ROMERO JUAN</t>
+        </is>
+      </c>
+      <c r="G43" s="1" t="inlineStr">
+        <is>
+          <t>ALBERTO LARA ROMERO JUAN</t>
+        </is>
+      </c>
+      <c r="H43" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I43" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="J43" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="K43" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="L43" s="1" t="n">
+        <v>1498</v>
+      </c>
+      <c r="M43" s="1" t="n">
+        <v>1498.01</v>
+      </c>
+      <c r="N43" s="1" t="inlineStr">
+        <is>
+          <t>17.9785091,-92.95955649999999</t>
+        </is>
+      </c>
+      <c r="O43" s="1" t="inlineStr">
+        <is>
+          <t>17.9785091,-92.95955649999999</t>
+        </is>
+      </c>
+      <c r="P43" s="1" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q43" s="1" t="inlineStr">
+        <is>
+          <t>SPRING_6457</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>SPRING</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>7034863026285</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>6456</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2025-11-27T09:02:44-06:00</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>CLAUDIA HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>CLAUDIA HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="H44" t="n">
+        <v>2</v>
+      </c>
+      <c r="I44" t="n">
+        <v>2</v>
+      </c>
+      <c r="J44" t="n">
+        <v>2</v>
+      </c>
+      <c r="K44" t="n">
+        <v>2</v>
+      </c>
+      <c r="L44" t="n">
+        <v>299</v>
+      </c>
+      <c r="M44" t="n">
+        <v>299.01</v>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>19.3927198,-99.0836971</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>19.3927198,-99.0836971</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>SPRING_6456</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>SPRING</t>
+        </is>
+      </c>
+      <c r="B45" s="1" t="inlineStr">
+        <is>
+          <t>7034328285293</t>
+        </is>
+      </c>
+      <c r="C45" s="1" t="inlineStr">
+        <is>
+          <t>6455</t>
+        </is>
+      </c>
+      <c r="D45" s="1" t="inlineStr">
+        <is>
+          <t>2025-11-27T03:19:50-06:00</t>
+        </is>
+      </c>
+      <c r="E45" s="1" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="F45" s="1" t="inlineStr">
+        <is>
+          <t>LAURA ALGARIN ORTEGA</t>
+        </is>
+      </c>
+      <c r="G45" s="1" t="inlineStr">
+        <is>
+          <t>LAURA ALGARIN ORTEGA</t>
+        </is>
+      </c>
+      <c r="H45" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I45" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="J45" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="K45" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L45" s="1" t="n">
+        <v>4749</v>
+      </c>
+      <c r="M45" s="1" t="n">
+        <v>4749.01</v>
+      </c>
+      <c r="N45" s="1" t="inlineStr">
+        <is>
+          <t>18.994729,-98.2796752</t>
+        </is>
+      </c>
+      <c r="O45" s="1" t="inlineStr">
+        <is>
+          <t>18.994729,-98.2796752</t>
+        </is>
+      </c>
+      <c r="P45" s="1" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q45" s="1" t="inlineStr">
+        <is>
+          <t>SPRING_6455</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>SPRING</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>7033865863277</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>6454</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>2025-11-27T01:06:27-06:00</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>MIGUEL MENA</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>MIGUEL MENA</t>
+        </is>
+      </c>
+      <c r="H46" t="n">
+        <v>2</v>
+      </c>
+      <c r="I46" t="n">
+        <v>2</v>
+      </c>
+      <c r="J46" t="n">
+        <v>2</v>
+      </c>
+      <c r="K46" t="n">
+        <v>2</v>
+      </c>
+      <c r="L46" t="n">
+        <v>4999</v>
+      </c>
+      <c r="M46" t="n">
+        <v>4999.01</v>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>23.4581588,-110.2273739</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>23.4581588,-110.2273739</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>SPRING_6454</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="inlineStr">
+        <is>
           <t>ATLAS</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>6092039880757</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>18854</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>2025-11-21T08:30:54-06:00</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>paid</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>LILIANA HERRERA MORALES</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>LILIANA HERRERA MORALES</t>
-        </is>
-      </c>
-      <c r="H42" t="n">
-        <v>1</v>
-      </c>
-      <c r="I42" t="n">
-        <v>1</v>
-      </c>
-      <c r="J42" t="n">
-        <v>1</v>
-      </c>
-      <c r="K42" t="n">
-        <v>1</v>
-      </c>
-      <c r="L42" t="n">
-        <v>2499</v>
-      </c>
-      <c r="M42" t="n">
-        <v>2499</v>
-      </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>18.6004478,-98.45628339999999</t>
-        </is>
-      </c>
-      <c r="O42" t="inlineStr">
-        <is>
-          <t>18.6004478,-98.45628339999999</t>
-        </is>
-      </c>
-      <c r="P42" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="Q42" t="inlineStr">
-        <is>
-          <t>ATLAS_18854</t>
+      <c r="B47" s="1" t="inlineStr">
+        <is>
+          <t>6106073956405</t>
+        </is>
+      </c>
+      <c r="C47" s="1" t="inlineStr">
+        <is>
+          <t>18989</t>
+        </is>
+      </c>
+      <c r="D47" s="1" t="inlineStr">
+        <is>
+          <t>2025-11-27T22:32:47-06:00</t>
+        </is>
+      </c>
+      <c r="E47" s="1" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="F47" s="1" t="inlineStr">
+        <is>
+          <t>TANIA MORALES CEDILLO</t>
+        </is>
+      </c>
+      <c r="G47" s="1" t="inlineStr">
+        <is>
+          <t>TANIA MORALES CEDILLO</t>
+        </is>
+      </c>
+      <c r="H47" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I47" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J47" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K47" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L47" s="1" t="n">
+        <v>13299.05</v>
+      </c>
+      <c r="M47" s="1" t="n">
+        <v>13299.05</v>
+      </c>
+      <c r="N47" s="1" t="inlineStr">
+        <is>
+          <t>19.2464833,-99.0753003</t>
+        </is>
+      </c>
+      <c r="O47" s="1" t="inlineStr">
+        <is>
+          <t>19.2464833,-99.0753003</t>
+        </is>
+      </c>
+      <c r="P47" s="1" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q47" s="1" t="inlineStr">
+        <is>
+          <t>ATLAS_18989</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>ATLAS</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>6105999999029</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>18988</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>2025-11-27T21:41:48-06:00</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>KARLA SEELIGER</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>KARLA SEELIGER</t>
+        </is>
+      </c>
+      <c r="H48" t="n">
+        <v>1</v>
+      </c>
+      <c r="I48" t="n">
+        <v>1</v>
+      </c>
+      <c r="J48" t="n">
+        <v>1</v>
+      </c>
+      <c r="K48" t="n">
+        <v>1</v>
+      </c>
+      <c r="L48" t="n">
+        <v>11699</v>
+      </c>
+      <c r="M48" t="n">
+        <v>11699</v>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>19.5466309,-99.2831425</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>19.5466309,-99.2831425</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>ATLAS_18988</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t>ATLAS</t>
+        </is>
+      </c>
+      <c r="B49" s="1" t="inlineStr">
+        <is>
+          <t>6105986891829</t>
+        </is>
+      </c>
+      <c r="C49" s="1" t="inlineStr">
+        <is>
+          <t>18987</t>
+        </is>
+      </c>
+      <c r="D49" s="1" t="inlineStr">
+        <is>
+          <t>2025-11-27T21:32:45-06:00</t>
+        </is>
+      </c>
+      <c r="E49" s="1" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="F49" s="1" t="inlineStr">
+        <is>
+          <t>ROSA  MARIA GUADALUPE SADALLAH PEREZ</t>
+        </is>
+      </c>
+      <c r="G49" s="1" t="inlineStr">
+        <is>
+          <t>ROSA  MARIA GUADALUPE SADALLAH PEREZ</t>
+        </is>
+      </c>
+      <c r="H49" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I49" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J49" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K49" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L49" s="1" t="n">
+        <v>7959</v>
+      </c>
+      <c r="M49" s="1" t="n">
+        <v>7959</v>
+      </c>
+      <c r="N49" s="1" t="inlineStr">
+        <is>
+          <t>19.4783276,-99.2369265</t>
+        </is>
+      </c>
+      <c r="O49" s="1" t="inlineStr">
+        <is>
+          <t>19.4783276,-99.2369265</t>
+        </is>
+      </c>
+      <c r="P49" s="1" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q49" s="1" t="inlineStr">
+        <is>
+          <t>ATLAS_18987</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>ATLAS</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>6105962053685</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>18986</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>2025-11-27T21:16:49-06:00</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>IRIS JOSELIN LEON</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>IRIS JOSELIN LEON</t>
+        </is>
+      </c>
+      <c r="H50" t="n">
+        <v>1</v>
+      </c>
+      <c r="I50" t="n">
+        <v>1</v>
+      </c>
+      <c r="J50" t="n">
+        <v>1</v>
+      </c>
+      <c r="K50" t="n">
+        <v>1</v>
+      </c>
+      <c r="L50" t="n">
+        <v>4131.55</v>
+      </c>
+      <c r="M50" t="n">
+        <v>4131.55</v>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>20.6074495,-100.4691637</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>20.6074495,-100.4691637</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>ATLAS_18986</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="inlineStr">
+        <is>
+          <t>ATLAS</t>
+        </is>
+      </c>
+      <c r="B51" s="1" t="inlineStr">
+        <is>
+          <t>6105700237365</t>
+        </is>
+      </c>
+      <c r="C51" s="1" t="inlineStr">
+        <is>
+          <t>18985</t>
+        </is>
+      </c>
+      <c r="D51" s="1" t="inlineStr">
+        <is>
+          <t>2025-11-27T19:41:36-06:00</t>
+        </is>
+      </c>
+      <c r="E51" s="1" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="F51" s="1" t="inlineStr">
+        <is>
+          <t>ABIMAEL DAMACIO</t>
+        </is>
+      </c>
+      <c r="G51" s="1" t="inlineStr">
+        <is>
+          <t>ABIMAEL DAMACIO</t>
+        </is>
+      </c>
+      <c r="H51" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I51" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J51" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K51" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L51" s="1" t="n">
+        <v>2879</v>
+      </c>
+      <c r="M51" s="1" t="n">
+        <v>2879</v>
+      </c>
+      <c r="N51" s="1" t="inlineStr">
+        <is>
+          <t>19.5975348,-99.04851420000001</t>
+        </is>
+      </c>
+      <c r="O51" s="1" t="inlineStr">
+        <is>
+          <t>19.5975348,-99.04851420000001</t>
+        </is>
+      </c>
+      <c r="P51" s="1" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q51" s="1" t="inlineStr">
+        <is>
+          <t>ATLAS_18985</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>ATLAS</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>6105678184501</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>18984</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>2025-11-27T19:27:39-06:00</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>LUCIA CORDOVA CASTILLO</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>LUCIA CORDOVA CASTILLO</t>
+        </is>
+      </c>
+      <c r="H52" t="n">
+        <v>2</v>
+      </c>
+      <c r="I52" t="n">
+        <v>2</v>
+      </c>
+      <c r="J52" t="n">
+        <v>2</v>
+      </c>
+      <c r="K52" t="n">
+        <v>2</v>
+      </c>
+      <c r="L52" t="n">
+        <v>3248</v>
+      </c>
+      <c r="M52" t="n">
+        <v>3248</v>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>18.0338124,-92.89887329999999</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>18.0338124,-92.89887329999999</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>ATLAS_18984</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="inlineStr">
+        <is>
+          <t>ATLAS</t>
+        </is>
+      </c>
+      <c r="B53" s="1" t="inlineStr">
+        <is>
+          <t>6105663242293</t>
+        </is>
+      </c>
+      <c r="C53" s="1" t="inlineStr">
+        <is>
+          <t>18983</t>
+        </is>
+      </c>
+      <c r="D53" s="1" t="inlineStr">
+        <is>
+          <t>2025-11-27T19:18:15-06:00</t>
+        </is>
+      </c>
+      <c r="E53" s="1" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="F53" s="1" t="inlineStr">
+        <is>
+          <t>KATHARINA ROEHR KIESSLING</t>
+        </is>
+      </c>
+      <c r="G53" s="1" t="inlineStr">
+        <is>
+          <t>KATHARINA ROEHR KIESSLING</t>
+        </is>
+      </c>
+      <c r="H53" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I53" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J53" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K53" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L53" s="1" t="n">
+        <v>4099</v>
+      </c>
+      <c r="M53" s="1" t="n">
+        <v>4099</v>
+      </c>
+      <c r="N53" s="1" t="inlineStr">
+        <is>
+          <t>19.4324884,-99.186623</t>
+        </is>
+      </c>
+      <c r="O53" s="1" t="inlineStr">
+        <is>
+          <t>19.4324884,-99.186623</t>
+        </is>
+      </c>
+      <c r="P53" s="1" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q53" s="1" t="inlineStr">
+        <is>
+          <t>ATLAS_18983</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ATLAS</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>6105613762613</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>18982</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>2025-11-27T18:49:08-06:00</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>JESÚS ADRIÁN SIERRA PERALTA</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>JESÚS ADRIÁN SIERRA PERALTA</t>
+        </is>
+      </c>
+      <c r="H54" t="n">
+        <v>1</v>
+      </c>
+      <c r="I54" t="n">
+        <v>1</v>
+      </c>
+      <c r="J54" t="n">
+        <v>1</v>
+      </c>
+      <c r="K54" t="n">
+        <v>1</v>
+      </c>
+      <c r="L54" t="n">
+        <v>8349</v>
+      </c>
+      <c r="M54" t="n">
+        <v>8349</v>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>19.477989,-99.05423719999999</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>19.477989,-99.05423719999999</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>ENCONTRADO DÍA SIGUIENTE</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>ATLAS_18982</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="inlineStr">
+        <is>
+          <t>ATLAS</t>
+        </is>
+      </c>
+      <c r="B55" s="1" t="inlineStr">
+        <is>
+          <t>6105597706293</t>
+        </is>
+      </c>
+      <c r="C55" s="1" t="inlineStr">
+        <is>
+          <t>18981</t>
+        </is>
+      </c>
+      <c r="D55" s="1" t="inlineStr">
+        <is>
+          <t>2025-11-27T18:40:47-06:00</t>
+        </is>
+      </c>
+      <c r="E55" s="1" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="F55" s="1" t="inlineStr">
+        <is>
+          <t>SAUL VARILLAS GONZALEZ</t>
+        </is>
+      </c>
+      <c r="G55" s="1" t="inlineStr">
+        <is>
+          <t>SAUL VARILLAS GONZALEZ</t>
+        </is>
+      </c>
+      <c r="H55" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I55" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J55" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K55" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L55" s="1" t="n">
+        <v>6199</v>
+      </c>
+      <c r="M55" s="1" t="n">
+        <v>6199</v>
+      </c>
+      <c r="N55" s="1" t="inlineStr">
+        <is>
+          <t>18.9055089,-96.9477517</t>
+        </is>
+      </c>
+      <c r="O55" s="1" t="inlineStr">
+        <is>
+          <t>18.9055089,-96.9477517</t>
+        </is>
+      </c>
+      <c r="P55" s="1" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q55" s="1" t="inlineStr">
+        <is>
+          <t>ATLAS_18981</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>ATLAS</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>6105581879349</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>18980</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>2025-11-27T18:33:28-06:00</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>ADMIN ESCAJAL</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>ADMIN ESCAJAL</t>
+        </is>
+      </c>
+      <c r="H56" t="n">
+        <v>1</v>
+      </c>
+      <c r="I56" t="n">
+        <v>1</v>
+      </c>
+      <c r="J56" t="n">
+        <v>1</v>
+      </c>
+      <c r="K56" t="n">
+        <v>1</v>
+      </c>
+      <c r="L56" t="n">
+        <v>6999</v>
+      </c>
+      <c r="M56" t="n">
+        <v>6999</v>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>19.3899039,-99.1517134</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>19.3899039,-99.1517134</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>ATLAS_18980</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="inlineStr">
+        <is>
+          <t>ATLAS</t>
+        </is>
+      </c>
+      <c r="B57" s="1" t="inlineStr">
+        <is>
+          <t>6105415581749</t>
+        </is>
+      </c>
+      <c r="C57" s="1" t="inlineStr">
+        <is>
+          <t>18979</t>
+        </is>
+      </c>
+      <c r="D57" s="1" t="inlineStr">
+        <is>
+          <t>2025-11-27T16:38:17-06:00</t>
+        </is>
+      </c>
+      <c r="E57" s="1" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="F57" s="1" t="inlineStr">
+        <is>
+          <t>NAYELI CORREA</t>
+        </is>
+      </c>
+      <c r="G57" s="1" t="inlineStr">
+        <is>
+          <t>NAYELI CORREA</t>
+        </is>
+      </c>
+      <c r="H57" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I57" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="J57" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K57" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L57" s="1" t="n">
+        <v>798</v>
+      </c>
+      <c r="M57" s="1" t="n">
+        <v>798</v>
+      </c>
+      <c r="N57" s="1" t="inlineStr">
+        <is>
+          <t>19.437185,-99.2567272</t>
+        </is>
+      </c>
+      <c r="O57" s="1" t="inlineStr">
+        <is>
+          <t>19.437185,-99.2567272</t>
+        </is>
+      </c>
+      <c r="P57" s="1" t="inlineStr">
+        <is>
+          <t>Cantidad dif (1.0 vs 2.0) | Registros dif (1 vs 2)</t>
+        </is>
+      </c>
+      <c r="Q57" s="1" t="inlineStr">
+        <is>
+          <t>ATLAS_18979</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>ATLAS</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>6105390743605</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>18978</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>2025-11-27T16:20:14-06:00</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>PAULA LIZBETH ALAMILLA</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>PAULA LIZBETH ALAMILLA</t>
+        </is>
+      </c>
+      <c r="H58" t="n">
+        <v>1</v>
+      </c>
+      <c r="I58" t="n">
+        <v>1</v>
+      </c>
+      <c r="J58" t="n">
+        <v>1</v>
+      </c>
+      <c r="K58" t="n">
+        <v>1</v>
+      </c>
+      <c r="L58" t="n">
+        <v>4199</v>
+      </c>
+      <c r="M58" t="n">
+        <v>4199</v>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>19.4029553,-99.06356459999999</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>19.4029553,-99.06356459999999</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>ATLAS_18978</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="inlineStr">
+        <is>
+          <t>ATLAS</t>
+        </is>
+      </c>
+      <c r="B59" s="1" t="inlineStr">
+        <is>
+          <t>6105341034549</t>
+        </is>
+      </c>
+      <c r="C59" s="1" t="inlineStr">
+        <is>
+          <t>18977</t>
+        </is>
+      </c>
+      <c r="D59" s="1" t="inlineStr">
+        <is>
+          <t>2025-11-27T15:45:07-06:00</t>
+        </is>
+      </c>
+      <c r="E59" s="1" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="F59" s="1" t="inlineStr">
+        <is>
+          <t>DIANA MENDOZA HERNÁNDEZ</t>
+        </is>
+      </c>
+      <c r="G59" s="1" t="inlineStr">
+        <is>
+          <t>DIANA MENDOZA HERNÁNDEZ</t>
+        </is>
+      </c>
+      <c r="H59" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I59" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="J59" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="K59" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L59" s="1" t="n">
+        <v>16053.1</v>
+      </c>
+      <c r="M59" s="1" t="n">
+        <v>16053.1</v>
+      </c>
+      <c r="N59" s="1" t="inlineStr">
+        <is>
+          <t>16.8008242,-95.0889262</t>
+        </is>
+      </c>
+      <c r="O59" s="1" t="inlineStr">
+        <is>
+          <t>16.8008242,-95.0889262</t>
+        </is>
+      </c>
+      <c r="P59" s="1" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q59" s="1" t="inlineStr">
+        <is>
+          <t>ATLAS_18977</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>ATLAS</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>6105218547765</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>18976</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>2025-11-27T14:29:20-06:00</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>CARMEN GARCIA MARTINEZ</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>CARMEN GARCIA MARTINEZ</t>
+        </is>
+      </c>
+      <c r="H60" t="n">
+        <v>1</v>
+      </c>
+      <c r="I60" t="n">
+        <v>1</v>
+      </c>
+      <c r="J60" t="n">
+        <v>1</v>
+      </c>
+      <c r="K60" t="n">
+        <v>1</v>
+      </c>
+      <c r="L60" t="n">
+        <v>6649.05</v>
+      </c>
+      <c r="M60" t="n">
+        <v>6649.05</v>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>19.6208273,-99.2548599</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>19.6208273,-99.2548599</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>ATLAS_18976</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="inlineStr">
+        <is>
+          <t>ATLAS</t>
+        </is>
+      </c>
+      <c r="B61" s="1" t="inlineStr">
+        <is>
+          <t>6105092522037</t>
+        </is>
+      </c>
+      <c r="C61" s="1" t="inlineStr">
+        <is>
+          <t>18975</t>
+        </is>
+      </c>
+      <c r="D61" s="1" t="inlineStr">
+        <is>
+          <t>2025-11-27T13:22:02-06:00</t>
+        </is>
+      </c>
+      <c r="E61" s="1" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="F61" s="1" t="inlineStr">
+        <is>
+          <t>YURITZI JOVANNA ALARCÓN ZEMPOALTECA</t>
+        </is>
+      </c>
+      <c r="G61" s="1" t="inlineStr">
+        <is>
+          <t>YURITZI JOVANNA ALARCÓN ZEMPOALTECA</t>
+        </is>
+      </c>
+      <c r="H61" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I61" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J61" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K61" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L61" s="1" t="n">
+        <v>10999</v>
+      </c>
+      <c r="M61" s="1" t="n">
+        <v>10999</v>
+      </c>
+      <c r="N61" s="1" t="inlineStr">
+        <is>
+          <t>19.4913627,-99.2026691</t>
+        </is>
+      </c>
+      <c r="O61" s="1" t="inlineStr">
+        <is>
+          <t>19.4913627,-99.2026691</t>
+        </is>
+      </c>
+      <c r="P61" s="1" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q61" s="1" t="inlineStr">
+        <is>
+          <t>ATLAS_18975</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>ATLAS</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>6104624103477</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>18974</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>2025-11-27T09:51:22-06:00</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>GABRIEL OMAR HERNANDEZ ESCAMPA ABARCA</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>GABRIEL OMAR HERNANDEZ ESCAMPA ABARCA</t>
+        </is>
+      </c>
+      <c r="H62" t="n">
+        <v>2</v>
+      </c>
+      <c r="I62" t="n">
+        <v>2</v>
+      </c>
+      <c r="J62" t="n">
+        <v>2</v>
+      </c>
+      <c r="K62" t="n">
+        <v>2</v>
+      </c>
+      <c r="L62" t="n">
+        <v>11825.6</v>
+      </c>
+      <c r="M62" t="n">
+        <v>11825.6</v>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>19.301232,-99.1067003</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>19.301232,-99.1067003</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>ATLAS_18974</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="inlineStr">
+        <is>
+          <t>ATLAS</t>
+        </is>
+      </c>
+      <c r="B63" s="1" t="inlineStr">
+        <is>
+          <t>6104616271925</t>
+        </is>
+      </c>
+      <c r="C63" s="1" t="inlineStr">
+        <is>
+          <t>18973</t>
+        </is>
+      </c>
+      <c r="D63" s="1" t="inlineStr">
+        <is>
+          <t>2025-11-27T09:46:22-06:00</t>
+        </is>
+      </c>
+      <c r="E63" s="1" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="F63" s="1" t="inlineStr">
+        <is>
+          <t>DANIEL HURTADO RIVERA</t>
+        </is>
+      </c>
+      <c r="G63" s="1" t="inlineStr">
+        <is>
+          <t>DANIEL HURTADO RIVERA</t>
+        </is>
+      </c>
+      <c r="H63" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I63" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J63" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K63" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L63" s="1" t="n">
+        <v>1649</v>
+      </c>
+      <c r="M63" s="1" t="n">
+        <v>1649</v>
+      </c>
+      <c r="N63" s="1" t="inlineStr">
+        <is>
+          <t>19.682043,-99.0982813</t>
+        </is>
+      </c>
+      <c r="O63" s="1" t="inlineStr">
+        <is>
+          <t>19.682043,-99.0982813</t>
+        </is>
+      </c>
+      <c r="P63" s="1" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q63" s="1" t="inlineStr">
+        <is>
+          <t>ATLAS_18973</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>ATLAS</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>6104467537973</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>18972</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>2025-11-27T08:09:22-06:00</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>MAYA GONZALEZ</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>MAYA GONZALEZ</t>
+        </is>
+      </c>
+      <c r="H64" t="n">
+        <v>1</v>
+      </c>
+      <c r="I64" t="n">
+        <v>1</v>
+      </c>
+      <c r="J64" t="n">
+        <v>1</v>
+      </c>
+      <c r="K64" t="n">
+        <v>1</v>
+      </c>
+      <c r="L64" t="n">
+        <v>5799</v>
+      </c>
+      <c r="M64" t="n">
+        <v>5799</v>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>19.5914364,-99.0069703</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>19.5914364,-99.0069703</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>ATLAS_18972</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="inlineStr">
+        <is>
+          <t>ATLAS</t>
+        </is>
+      </c>
+      <c r="B65" s="1" t="inlineStr">
+        <is>
+          <t>6104252055605</t>
+        </is>
+      </c>
+      <c r="C65" s="1" t="inlineStr">
+        <is>
+          <t>18971</t>
+        </is>
+      </c>
+      <c r="D65" s="1" t="inlineStr">
+        <is>
+          <t>2025-11-27T05:01:59-06:00</t>
+        </is>
+      </c>
+      <c r="E65" s="1" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="F65" s="1" t="inlineStr">
+        <is>
+          <t>JAVIER ISAAC AGUIRRE BAUTISTA</t>
+        </is>
+      </c>
+      <c r="G65" s="1" t="inlineStr">
+        <is>
+          <t>JAVIER ISAAC AGUIRRE BAUTISTA</t>
+        </is>
+      </c>
+      <c r="H65" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I65" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J65" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K65" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L65" s="1" t="n">
+        <v>4199</v>
+      </c>
+      <c r="M65" s="1" t="n">
+        <v>4199</v>
+      </c>
+      <c r="N65" s="1" t="inlineStr">
+        <is>
+          <t>19.3117042,-99.1563126</t>
+        </is>
+      </c>
+      <c r="O65" s="1" t="inlineStr">
+        <is>
+          <t>19.3117042,-99.1563126</t>
+        </is>
+      </c>
+      <c r="P65" s="1" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q65" s="1" t="inlineStr">
+        <is>
+          <t>ATLAS_18971</t>
         </is>
       </c>
     </row>

</xml_diff>